<commit_message>
feat: add manual aluminum batch totals
Purpose:
- 让批量模板/API 支持逐炉手工铝块 kg/t，解决 API 导出与后台含 AH 铝块回算口径不一致的问题。
- 保持 LP 自动优化仍不投铝块，只在导出总消耗和总成本中单独计入现场铝块。

Changes:
- 在 01_批量任务 增加可选 手工铝块kg/t 字段，并在模板中补充铝块物料、价格示例和填写说明。
- 模板解析新增任务级 manualAluminum，按当前价格方案下铝块价格计算手工铝块成本；缺价时预检报错。
- 批量导出新增自动成本/消耗、手工铝块成本/用量、总成本/总消耗和炉次总成本列，并在路线明细追加手工录入铝块行。
- 新增解析和导出测试，更新 readme.md 与 issue_log.md，重新生成 alloy-batch-template-v1.xlsx。

Validation:
- .venv-win\\Scripts\\python.exe -m pytest tests\\test_batch_template.py -q
- .venv-win\\Scripts\\python.exe -m pytest tests\\test_backend_optimizer.py tests\\test_rule_engine.py tests\\test_batch_template.py -q
- node --test tests\\ui_static.test.js
- 使用正确版 workbook 填充新模板并通过 /api/template/validate、/api/batch-optimize、/api/batch-result 导出，328/328 成功。
- 运行 tools\\recalculate_lp_actual_aluminum.py 后与 API 含手工铝块总成本/总消耗对比，328 行差异计数为 0，最大误差约 5e-7。

Notes:
- 旧模板未填写 手工铝块kg/t 时仍按 0 处理，保持向后兼容。
- 工作区存在未纳入本提交的既有 AGENTS.md、outputs 删除/修改、Office 临时文件和 smoke 输出目录。
</commit_message>
<xml_diff>
--- a/alloy-batch-template-v1.xlsx
+++ b/alloy-batch-template-v1.xlsx
@@ -16,12 +16,12 @@
     <sheet name="07_工艺规则参数" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_批量任务'!$A$1:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_批量任务'!$A$1:$H$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_目标成分上下限'!$A$1:$U$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_转炉终点与回收率'!$A$1:$AL$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_合金成分库'!$A$1:$X$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_价格表'!$A$1:$D$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'06_填写说明与校验规则'!$A$1:$B$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_合金成分库'!$A$1:$X$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_价格表'!$A$1:$D$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'06_填写说明与校验规则'!$A$1:$B$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'07_工艺规则参数'!$A$1:$D$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -451,7 +451,8 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -487,6 +488,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>手工铝块kg/t</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>备注</t>
         </is>
       </c>
@@ -518,7 +524,8 @@
           <t>Q235B-1</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>正常样例，可复制新增任务</t>
         </is>
@@ -551,14 +558,15 @@
           <t>Q355C-1</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>批量任务互不影响</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G3"/>
+  <autoFilter ref="A1:H3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1199,7 +1207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X8"/>
+  <dimension ref="A1:X9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1225,7 +1233,7 @@
     <col width="10" customWidth="1" min="21" max="21"/>
     <col width="10" customWidth="1" min="22" max="22"/>
     <col width="28" customWidth="1" min="23" max="23"/>
-    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1730,8 +1738,66 @@
       <c r="W8" s="2" t="n"/>
       <c r="X8" s="2" t="inlineStr"/>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>铝块</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>铝块</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>连续</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="2" t="n"/>
+      <c r="M9" s="2" t="n"/>
+      <c r="N9" s="2" t="n"/>
+      <c r="O9" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="P9" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="Q9" s="2" t="n"/>
+      <c r="R9" s="2" t="n"/>
+      <c r="S9" s="2" t="n"/>
+      <c r="T9" s="2" t="n"/>
+      <c r="U9" s="2" t="n"/>
+      <c r="V9" s="2" t="n"/>
+      <c r="W9" s="2" t="n"/>
+      <c r="X9" s="2" t="inlineStr">
+        <is>
+          <t>手工铝块按 01_批量任务 的手工铝块kg/t 单独计入，不参与 LP 自动优化。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:X8"/>
+  <autoFilter ref="A1:X9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1742,7 +1808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1913,8 +1979,28 @@
         <v>14956</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>铝块</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>22337</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D8"/>
+  <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1925,7 +2011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1995,101 +2081,113 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>合金用量公式</t>
+          <t>手工铝块</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>kg/t = (目标成分 - 有效终点成分) / 合金品位 / 回收率 * 1000；当前批量链路只使用 C/Mn 终点扣减，V/Nb/Ti/Cr 等不做终点残余扣减；26MnB5 的 Si 回收率若录成 0 会按现场确认值 0.8 修正。</t>
+          <t>01_批量任务 可填写 手工铝块kg/t；该值不参与 LP 自动优化，只在批量导出时按铝块价格单独计入总合金消耗和总吨钢成本。空值或 0 表示本炉不单独计入铝块。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>标准元素</t>
+          <t>合金用量公式</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>标准模板仅保留 C, Si, Mn, P, S, V, Nb, Ti, Als, Alt, Ca, Cr, Ni, Cu, Mo, B, Sb；旧模板里的 N 上传时会被忽略。</t>
+          <t>kg/t = (目标成分 - 有效终点成分) / 合金品位 / 回收率 * 1000；当前批量链路只使用 C/Mn 终点扣减，V/Nb/Ti/Cr 等不做终点残余扣减；26MnB5 的 Si 回收率若录成 0 会按现场确认值 0.8 修正。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>P/S 规则</t>
+          <t>标准元素</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>P/S 通常只填写上限；转炉终点已超过上限时任务直接失败。</t>
+          <t>标准模板仅保留 C, Si, Mn, P, S, V, Nb, Ti, Als, Alt, Ca, Cr, Ni, Cu, Mo, B, Sb；旧模板里的 N 上传时会被忽略。</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>投料方式</t>
+          <t>P/S 规则</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>投料方式只能填写 连续 或 整袋；连续物料袋重kg留空或填 0，整袋物料袋重kg必须大于 0。</t>
+          <t>P/S 通常只填写上限；转炉终点已超过上限时任务直接失败。</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>路线序号</t>
+          <t>投料方式</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>最优路线明细中的路线序号只表示导出排序，从 1 开始，按成本贡献降序排列；它不是现场真实投料顺序。</t>
+          <t>投料方式只能填写 连续 或 整袋；连续物料袋重kg留空或填 0，整袋物料袋重kg必须大于 0。</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>规则参数</t>
+          <t>路线序号</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>07_工艺规则参数 是可编辑业务 sheet；修改阈值后，预检通过的批量任务会按该 sheet 中的规则求解。</t>
+          <t>最优路线明细中的路线序号只表示导出排序，从 1 开始，按成本贡献降序排列；它不是现场真实投料顺序。</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>禁止内容</t>
+          <t>规则参数</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>业务输入区不允许合并单元格、公式、空表头、重复表头、隐藏必填列。</t>
+          <t>07_工艺规则参数 是可编辑业务 sheet；修改阈值后，预检通过的批量任务会按该 sheet 中的规则求解。</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>禁止内容</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>业务输入区不允许合并单元格、公式、空表头、重复表头、隐藏必填列。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>错误定位</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>系统会返回 sheet、行号、字段、错误码、原因和修正建议。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B13"/>
+  <autoFilter ref="A1:B14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>